<commit_message>
second to last sheet implementation
</commit_message>
<xml_diff>
--- a/output/IMG_9693.xlsx
+++ b/output/IMG_9693.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="基準客先別シンプルリスト" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="2026年2月　　　　　　　　　　　　　　　基準客先別シンプ" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -61,7 +61,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="64">
+  <borders count="76">
     <border>
       <left/>
       <right/>
@@ -89,6 +89,38 @@
     </border>
     <border>
       <left style="thin"/>
+      <right style="thin">
+        <color rgb="00D9D9D9"/>
+      </right>
+      <top style="medium"/>
+      <bottom/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin">
+        <color rgb="00D9D9D9"/>
+      </right>
+      <top/>
+      <bottom style="medium"/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00D9D9D9"/>
+      </left>
+      <right style="thin"/>
+      <top style="medium"/>
+      <bottom/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00D9D9D9"/>
+      </left>
+      <right style="thin"/>
+      <top/>
+      <bottom style="medium"/>
+    </border>
+    <border>
+      <left style="thin"/>
       <right style="thin"/>
       <top style="medium"/>
       <bottom/>
@@ -133,6 +165,18 @@
     </border>
     <border>
       <left style="medium"/>
+      <right style="thin">
+        <color rgb="00FFFFFF"/>
+      </right>
+      <top style="medium"/>
+      <bottom style="thin">
+        <color rgb="00FFFFFF"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00FFFFFF"/>
+      </left>
       <right style="medium"/>
       <top style="medium"/>
       <bottom style="thin">
@@ -181,6 +225,20 @@
     </border>
     <border>
       <left style="medium"/>
+      <right style="thin">
+        <color rgb="00FFFFFF"/>
+      </right>
+      <top style="thin">
+        <color rgb="00FFFFFF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00FFFFFF"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00FFFFFF"/>
+      </left>
       <right style="medium"/>
       <top style="thin">
         <color rgb="00FFFFFF"/>
@@ -259,6 +317,18 @@
     </border>
     <border>
       <left style="medium"/>
+      <right style="thin">
+        <color rgb="00FFFFFF"/>
+      </right>
+      <top style="thin">
+        <color rgb="00FFFFFF"/>
+      </top>
+      <bottom style="medium"/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00FFFFFF"/>
+      </left>
       <right style="medium"/>
       <top style="thin">
         <color rgb="00FFFFFF"/>
@@ -281,6 +351,18 @@
     </border>
     <border>
       <left style="medium"/>
+      <right style="thin">
+        <color rgb="00D9D9D9"/>
+      </right>
+      <top style="medium"/>
+      <bottom style="thin">
+        <color rgb="00D9D9D9"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00D9D9D9"/>
+      </left>
       <right style="medium"/>
       <top style="medium"/>
       <bottom style="thin">
@@ -323,6 +405,20 @@
     </border>
     <border>
       <left style="medium"/>
+      <right style="thin">
+        <color rgb="00D9D9D9"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D9D9D9"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D9D9D9"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00D9D9D9"/>
+      </left>
       <right style="medium"/>
       <top style="thin">
         <color rgb="00D9D9D9"/>
@@ -395,6 +491,18 @@
     </border>
     <border>
       <left style="medium"/>
+      <right style="thin">
+        <color rgb="00D9D9D9"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D9D9D9"/>
+      </top>
+      <bottom style="medium"/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00D9D9D9"/>
+      </left>
       <right style="medium"/>
       <top style="thin">
         <color rgb="00D9D9D9"/>
@@ -411,6 +519,18 @@
     </border>
     <border>
       <left style="medium"/>
+      <right style="thin">
+        <color rgb="00D9D9D9"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D9D9D9"/>
+      </top>
+      <bottom style="thick"/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00D9D9D9"/>
+      </left>
       <right style="medium"/>
       <top style="thin">
         <color rgb="00D9D9D9"/>
@@ -483,6 +603,18 @@
     </border>
     <border>
       <left style="medium"/>
+      <right style="thin">
+        <color rgb="00FFFFFF"/>
+      </right>
+      <top style="thick"/>
+      <bottom style="thin">
+        <color rgb="00FFFFFF"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00FFFFFF"/>
+      </left>
       <right style="medium"/>
       <top style="thick"/>
       <bottom style="thin">
@@ -575,7 +707,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="68">
+  <cellXfs count="80">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -598,6 +730,12 @@
     <xf numFmtId="0" fontId="4" fillId="2" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -610,166 +748,196 @@
     <xf numFmtId="0" fontId="4" fillId="2" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="16" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="16" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="19" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="22" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="23" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="19" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="22" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="23" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="26" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="27" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="28" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="29" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="30" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="31" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="27" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="32" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="33" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="34" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="28" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="29" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="35" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="36" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="37" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="30" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="31" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="32" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="33" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="34" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="38" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="39" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="40" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="41" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="35" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="36" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="37" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="38" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="39" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="40" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="41" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="42" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="43" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="44" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="45" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="46" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="47" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="48" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="49" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="50" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="45" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="51" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="52" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="53" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="54" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="55" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="56" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="46" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="47" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="48" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="49" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="53" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="57" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="58" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="59" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="60" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="64" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="54" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="65" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="66" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="55" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="56" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="57" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="50" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="58" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="59" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="51" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="60" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="61" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="62" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="52" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="63" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="67" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="68" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="69" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="61" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="70" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="71" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="62" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="72" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="73" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="74" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="63" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="75" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1137,24 +1305,25 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O27"/>
+  <dimension ref="A1:P27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="9.1" customWidth="1" min="1" max="1"/>
-    <col width="58.15" customWidth="1" min="2" max="2"/>
-    <col width="6.74" customWidth="1" min="3" max="3"/>
-    <col width="17.25" customWidth="1" min="4" max="4"/>
-    <col width="12.05" customWidth="1" min="5" max="5"/>
-    <col width="18.2" customWidth="1" min="6" max="6"/>
-    <col width="13" customWidth="1" min="7" max="7"/>
-    <col width="16.55" customWidth="1" min="8" max="8"/>
-    <col width="13" customWidth="1" min="9" max="9"/>
-    <col width="13" customWidth="1" min="10" max="10"/>
-    <col width="13" customWidth="1" min="11" max="11"/>
-    <col width="13" customWidth="1" min="12" max="12"/>
-    <col width="15.36" customWidth="1" min="13" max="13"/>
-    <col width="16.55" customWidth="1" min="14" max="14"/>
-    <col width="18.2" customWidth="1" min="15" max="15"/>
+    <col width="9.800000000000001" customWidth="1" min="1" max="1"/>
+    <col width="31.43" customWidth="1" min="2" max="2"/>
+    <col width="31.31" customWidth="1" min="3" max="3"/>
+    <col width="7.26" customWidth="1" min="4" max="4"/>
+    <col width="18.58" customWidth="1" min="5" max="5"/>
+    <col width="12.98" customWidth="1" min="6" max="6"/>
+    <col width="19.6" customWidth="1" min="7" max="7"/>
+    <col width="17" customWidth="1" min="8" max="8"/>
+    <col width="17.82" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="13" max="13"/>
+    <col width="16.54" customWidth="1" min="14" max="14"/>
+    <col width="17.82" customWidth="1" min="15" max="15"/>
+    <col width="19.6" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1" ht="14" customHeight="1">
@@ -1165,12 +1334,12 @@
       </c>
       <c r="B1" s="1" t="n"/>
       <c r="C1" s="1" t="n"/>
-      <c r="D1" s="2" t="inlineStr">
+      <c r="D1" s="1" t="n"/>
+      <c r="E1" s="2" t="inlineStr">
         <is>
           <t>基準客先別シンプルリスト</t>
         </is>
       </c>
-      <c r="E1" s="2" t="n"/>
       <c r="F1" s="2" t="n"/>
       <c r="G1" s="2" t="n"/>
       <c r="H1" s="2" t="n"/>
@@ -1178,13 +1347,14 @@
       <c r="J1" s="2" t="n"/>
       <c r="K1" s="2" t="n"/>
       <c r="L1" s="2" t="n"/>
-      <c r="M1" s="3" t="inlineStr">
-        <is>
-          <t>2026/6/22 1</t>
-        </is>
-      </c>
-      <c r="N1" s="3" t="n"/>
+      <c r="M1" s="2" t="n"/>
+      <c r="N1" s="3" t="inlineStr">
+        <is>
+          <t>2026/6/22 PAGE:1</t>
+        </is>
+      </c>
       <c r="O1" s="3" t="n"/>
+      <c r="P1" s="3" t="n"/>
     </row>
     <row r="2" ht="14" customHeight="1">
       <c r="A2" s="4" t="n"/>
@@ -1193,1365 +1363,1505 @@
           <t>基準客先</t>
         </is>
       </c>
-      <c r="C2" s="5" t="n"/>
-      <c r="D2" s="6" t="inlineStr">
+      <c r="C2" s="6" t="n"/>
+      <c r="D2" s="7" t="n"/>
+      <c r="E2" s="8" t="inlineStr">
         <is>
           <t>営業粗利額</t>
         </is>
       </c>
-      <c r="E2" s="6" t="inlineStr">
+      <c r="F2" s="8" t="inlineStr">
         <is>
           <t>粗利率</t>
         </is>
       </c>
-      <c r="F2" s="6" t="inlineStr">
+      <c r="G2" s="8" t="inlineStr">
         <is>
           <t>純売上額</t>
         </is>
       </c>
-      <c r="G2" s="6" t="inlineStr">
+      <c r="H2" s="8" t="inlineStr">
         <is>
           <t>上進預り＋正式買品</t>
         </is>
       </c>
-      <c r="H2" s="6" t="inlineStr">
+      <c r="I2" s="8" t="inlineStr">
         <is>
           <t>本部売上</t>
         </is>
       </c>
-      <c r="I2" s="6" t="inlineStr">
+      <c r="J2" s="8" t="inlineStr">
         <is>
           <t>デザイン経費</t>
         </is>
       </c>
-      <c r="J2" s="6" t="inlineStr">
+      <c r="K2" s="8" t="inlineStr">
         <is>
           <t>在庫額</t>
         </is>
       </c>
-      <c r="K2" s="6" t="inlineStr">
+      <c r="L2" s="8" t="inlineStr">
         <is>
           <t>死蔵品額</t>
         </is>
       </c>
-      <c r="L2" s="6" t="inlineStr">
+      <c r="M2" s="8" t="inlineStr">
         <is>
           <t>印字仕入額</t>
         </is>
       </c>
-      <c r="M2" s="6" t="inlineStr">
+      <c r="N2" s="8" t="inlineStr">
         <is>
           <t>発送件数</t>
         </is>
       </c>
-      <c r="N2" s="6" t="inlineStr">
+      <c r="O2" s="8" t="inlineStr">
         <is>
           <t>物流経費</t>
         </is>
       </c>
-      <c r="O2" s="7" t="n"/>
+      <c r="P2" s="9" t="inlineStr">
+        <is>
+          <t>目標粗利額</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="14" customHeight="1">
-      <c r="A3" s="8" t="n"/>
-      <c r="B3" s="9" t="n"/>
-      <c r="C3" s="9" t="n"/>
-      <c r="D3" s="10" t="inlineStr">
+      <c r="A3" s="10" t="n"/>
+      <c r="B3" s="11" t="n"/>
+      <c r="C3" s="12" t="n"/>
+      <c r="D3" s="13" t="n"/>
+      <c r="E3" s="14" t="inlineStr">
         <is>
           <t>粗利達成率</t>
         </is>
       </c>
-      <c r="E3" s="10" t="inlineStr">
+      <c r="F3" s="14" t="inlineStr">
         <is>
           <t>可処率</t>
         </is>
       </c>
-      <c r="F3" s="10" t="inlineStr">
+      <c r="G3" s="14" t="inlineStr">
         <is>
           <t>売上達成率</t>
         </is>
       </c>
-      <c r="G3" s="10" t="inlineStr">
+      <c r="H3" s="14" t="inlineStr">
         <is>
           <t>上海扱い分の割合</t>
         </is>
       </c>
-      <c r="H3" s="10" t="inlineStr">
+      <c r="I3" s="14" t="inlineStr">
         <is>
           <t>緑資認裁粗利率</t>
         </is>
       </c>
-      <c r="I3" s="10" t="inlineStr">
+      <c r="J3" s="14" t="inlineStr">
         <is>
           <t>品質検査経費</t>
         </is>
       </c>
-      <c r="J3" s="10" t="inlineStr">
+      <c r="K3" s="14" t="inlineStr">
         <is>
           <t>在庫準備期間</t>
         </is>
       </c>
-      <c r="K3" s="10" t="inlineStr">
+      <c r="L3" s="14" t="inlineStr">
         <is>
           <t>死蔵品比率</t>
         </is>
       </c>
-      <c r="L3" s="10" t="inlineStr">
+      <c r="M3" s="14" t="inlineStr">
         <is>
           <t>印字仕入数</t>
         </is>
       </c>
-      <c r="M3" s="10" t="inlineStr">
+      <c r="N3" s="14" t="inlineStr">
         <is>
           <t>運賃</t>
         </is>
       </c>
-      <c r="N3" s="10" t="inlineStr">
+      <c r="O3" s="14" t="inlineStr">
         <is>
           <t>システム経費</t>
         </is>
       </c>
-      <c r="O3" s="11" t="inlineStr">
+      <c r="P3" s="15" t="inlineStr">
         <is>
           <t>目標売上額</t>
         </is>
       </c>
     </row>
     <row r="4" ht="13" customHeight="1">
-      <c r="A4" s="12" t="inlineStr">
+      <c r="A4" s="16" t="inlineStr">
         <is>
           <t>シ50</t>
         </is>
       </c>
-      <c r="B4" s="13" t="inlineStr">
+      <c r="B4" s="17" t="inlineStr">
+        <is>
+          <t>(株)ジュン</t>
+        </is>
+      </c>
+      <c r="C4" s="18" t="n"/>
+      <c r="D4" s="19" t="inlineStr">
         <is>
           <t>当月</t>
         </is>
       </c>
-      <c r="C4" s="14" t="inlineStr">
-        <is>
-          <t>当月</t>
-        </is>
-      </c>
-      <c r="D4" s="15" t="inlineStr">
+      <c r="E4" s="20" t="inlineStr">
         <is>
           <t>6,008,094</t>
         </is>
       </c>
-      <c r="E4" s="16" t="inlineStr">
+      <c r="F4" s="21" t="inlineStr">
         <is>
           <t>35.3</t>
         </is>
       </c>
-      <c r="F4" s="16" t="inlineStr">
+      <c r="G4" s="21" t="inlineStr">
         <is>
           <t>17,024,012</t>
         </is>
       </c>
-      <c r="G4" s="16" t="inlineStr">
+      <c r="H4" s="21" t="inlineStr">
         <is>
           <t>8,500,080</t>
         </is>
       </c>
-      <c r="H4" s="16" t="inlineStr">
+      <c r="I4" s="21" t="inlineStr">
         <is>
           <t>104,736</t>
         </is>
       </c>
-      <c r="I4" s="16" t="inlineStr">
+      <c r="J4" s="21" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="J4" s="16" t="inlineStr">
+      <c r="K4" s="21" t="inlineStr">
         <is>
           <t>31,270,029</t>
         </is>
       </c>
-      <c r="K4" s="16" t="inlineStr">
+      <c r="L4" s="21" t="inlineStr">
         <is>
           <t>362,832</t>
         </is>
       </c>
-      <c r="L4" s="16" t="inlineStr">
+      <c r="M4" s="21" t="inlineStr">
         <is>
           <t>2,519,776</t>
         </is>
       </c>
-      <c r="M4" s="16" t="inlineStr">
+      <c r="N4" s="21" t="inlineStr">
         <is>
           <t>483</t>
         </is>
       </c>
-      <c r="N4" s="16" t="inlineStr">
+      <c r="O4" s="21" t="inlineStr">
         <is>
           <t>411,042</t>
         </is>
       </c>
-      <c r="O4" s="17" t="inlineStr">
+      <c r="P4" s="22" t="inlineStr">
         <is>
           <t>8,984,250</t>
         </is>
       </c>
     </row>
     <row r="5" ht="13" customHeight="1">
-      <c r="A5" s="18" t="n"/>
-      <c r="B5" s="19" t="n"/>
-      <c r="C5" s="20" t="n"/>
-      <c r="D5" s="21" t="inlineStr">
+      <c r="A5" s="23" t="n"/>
+      <c r="B5" s="24" t="inlineStr">
+        <is>
+          <t>実績粗利     115,407,750 率 34</t>
+        </is>
+      </c>
+      <c r="C5" s="25" t="inlineStr">
+        <is>
+          <t>実績売上     339,753,881</t>
+        </is>
+      </c>
+      <c r="D5" s="26" t="n"/>
+      <c r="E5" s="27" t="inlineStr">
         <is>
           <t>66.9</t>
         </is>
       </c>
-      <c r="E5" s="22" t="n"/>
-      <c r="F5" s="22" t="inlineStr">
+      <c r="F5" s="28" t="n"/>
+      <c r="G5" s="28" t="inlineStr">
         <is>
           <t>68.8</t>
         </is>
       </c>
-      <c r="G5" s="22" t="inlineStr">
+      <c r="H5" s="28" t="inlineStr">
         <is>
           <t>49.9</t>
         </is>
       </c>
-      <c r="H5" s="22" t="n"/>
-      <c r="I5" s="22" t="n"/>
-      <c r="J5" s="22" t="inlineStr">
+      <c r="I5" s="28" t="n"/>
+      <c r="J5" s="28" t="n"/>
+      <c r="K5" s="28" t="inlineStr">
         <is>
           <t>2.7</t>
         </is>
       </c>
-      <c r="K5" s="22" t="inlineStr">
+      <c r="L5" s="28" t="inlineStr">
         <is>
           <t>3.9</t>
         </is>
       </c>
-      <c r="L5" s="22" t="inlineStr">
+      <c r="M5" s="28" t="inlineStr">
         <is>
           <t>674,476</t>
         </is>
       </c>
-      <c r="M5" s="22" t="inlineStr">
+      <c r="N5" s="28" t="inlineStr">
         <is>
           <t>609,174</t>
         </is>
       </c>
-      <c r="N5" s="22" t="inlineStr">
+      <c r="O5" s="28" t="inlineStr">
         <is>
           <t>93,840</t>
         </is>
       </c>
-      <c r="O5" s="23" t="inlineStr">
+      <c r="P5" s="29" t="inlineStr">
         <is>
           <t>24,750,000</t>
         </is>
       </c>
     </row>
     <row r="6" ht="13" customHeight="1">
-      <c r="A6" s="18" t="n"/>
-      <c r="B6" s="19" t="inlineStr">
+      <c r="A6" s="23" t="n"/>
+      <c r="B6" s="24" t="inlineStr">
+        <is>
+          <t>目標粗利     123,500,000 率 36</t>
+        </is>
+      </c>
+      <c r="C6" s="25" t="inlineStr">
+        <is>
+          <t>目標売上     340,000,000</t>
+        </is>
+      </c>
+      <c r="D6" s="26" t="inlineStr">
         <is>
           <t>累計</t>
         </is>
       </c>
-      <c r="C6" s="20" t="inlineStr">
-        <is>
-          <t>累計</t>
-        </is>
-      </c>
-      <c r="D6" s="24" t="inlineStr">
+      <c r="E6" s="30" t="inlineStr">
         <is>
           <t>102,967,486</t>
         </is>
       </c>
-      <c r="E6" s="25" t="inlineStr">
+      <c r="F6" s="31" t="inlineStr">
         <is>
           <t>35.8</t>
         </is>
       </c>
-      <c r="F6" s="25" t="inlineStr">
+      <c r="G6" s="31" t="inlineStr">
         <is>
           <t>287,650,236</t>
         </is>
       </c>
-      <c r="G6" s="25" t="inlineStr">
+      <c r="H6" s="31" t="inlineStr">
         <is>
           <t>182,124,664</t>
         </is>
       </c>
-      <c r="H6" s="25" t="inlineStr">
+      <c r="I6" s="31" t="inlineStr">
         <is>
           <t>1,118,068</t>
         </is>
       </c>
-      <c r="I6" s="25" t="inlineStr">
+      <c r="J6" s="31" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="J6" s="25" t="inlineStr">
+      <c r="K6" s="31" t="inlineStr">
         <is>
           <t>27,410,622</t>
         </is>
       </c>
-      <c r="K6" s="25" t="inlineStr">
+      <c r="L6" s="31" t="inlineStr">
         <is>
           <t>463,398</t>
         </is>
       </c>
-      <c r="L6" s="25" t="inlineStr">
+      <c r="M6" s="31" t="inlineStr">
         <is>
           <t>35,835,714</t>
         </is>
       </c>
-      <c r="M6" s="25" t="inlineStr">
+      <c r="N6" s="31" t="inlineStr">
         <is>
           <t>6,601</t>
         </is>
       </c>
-      <c r="N6" s="25" t="inlineStr">
+      <c r="O6" s="31" t="inlineStr">
         <is>
           <t>5,135,954</t>
         </is>
       </c>
-      <c r="O6" s="26" t="inlineStr">
+      <c r="P6" s="32" t="inlineStr">
         <is>
           <t>113,074,640</t>
         </is>
       </c>
     </row>
     <row r="7" ht="13" customHeight="1">
-      <c r="A7" s="27" t="n"/>
-      <c r="B7" s="28" t="n"/>
-      <c r="C7" s="29" t="n"/>
-      <c r="D7" s="21" t="inlineStr">
+      <c r="A7" s="33" t="n"/>
+      <c r="B7" s="34" t="n"/>
+      <c r="C7" s="35" t="inlineStr">
+        <is>
+          <t>目標在庫     28,000,000</t>
+        </is>
+      </c>
+      <c r="D7" s="36" t="n"/>
+      <c r="E7" s="27" t="inlineStr">
         <is>
           <t>91.1</t>
         </is>
       </c>
-      <c r="E7" s="22" t="inlineStr">
+      <c r="F7" s="28" t="inlineStr">
         <is>
           <t>34.6</t>
         </is>
       </c>
-      <c r="F7" s="22" t="inlineStr">
+      <c r="G7" s="28" t="inlineStr">
         <is>
           <t>92.4</t>
         </is>
       </c>
-      <c r="G7" s="22" t="inlineStr">
+      <c r="H7" s="28" t="inlineStr">
         <is>
           <t>63.3</t>
         </is>
       </c>
-      <c r="H7" s="22" t="n"/>
-      <c r="I7" s="22" t="n"/>
-      <c r="J7" s="22" t="inlineStr">
+      <c r="I7" s="28" t="n"/>
+      <c r="J7" s="28" t="n"/>
+      <c r="K7" s="28" t="inlineStr">
         <is>
           <t>0.0</t>
         </is>
       </c>
-      <c r="K7" s="22" t="n"/>
-      <c r="L7" s="22" t="inlineStr">
+      <c r="L7" s="28" t="n"/>
+      <c r="M7" s="28" t="inlineStr">
         <is>
           <t>10,973,554</t>
         </is>
       </c>
-      <c r="M7" s="22" t="inlineStr">
+      <c r="N7" s="28" t="inlineStr">
         <is>
           <t>12,086,717</t>
         </is>
       </c>
-      <c r="N7" s="22" t="inlineStr">
+      <c r="O7" s="28" t="inlineStr">
         <is>
           <t>1,881,400</t>
         </is>
       </c>
-      <c r="O7" s="23" t="inlineStr">
+      <c r="P7" s="29" t="inlineStr">
         <is>
           <t>311,280,000</t>
         </is>
       </c>
     </row>
     <row r="8" ht="13" customHeight="1">
-      <c r="A8" s="30" t="inlineStr">
-        <is>
-          <t>シ50
-元決済</t>
-        </is>
-      </c>
-      <c r="B8" s="31" t="inlineStr">
+      <c r="A8" s="37" t="inlineStr">
+        <is>
+          <t>シ50</t>
+        </is>
+      </c>
+      <c r="B8" s="38" t="inlineStr">
+        <is>
+          <t>(株)ジュン</t>
+        </is>
+      </c>
+      <c r="C8" s="39" t="n"/>
+      <c r="D8" s="40" t="inlineStr">
         <is>
           <t>当月</t>
         </is>
       </c>
-      <c r="C8" s="32" t="inlineStr">
-        <is>
-          <t>当月</t>
-        </is>
-      </c>
-      <c r="D8" s="33" t="inlineStr">
+      <c r="E8" s="41" t="inlineStr">
         <is>
           <t>1,436,915</t>
         </is>
       </c>
-      <c r="E8" s="34" t="inlineStr">
+      <c r="F8" s="42" t="inlineStr">
         <is>
           <t>44.4</t>
         </is>
       </c>
-      <c r="F8" s="34" t="inlineStr">
+      <c r="G8" s="42" t="inlineStr">
         <is>
           <t>3,234,127</t>
         </is>
       </c>
-      <c r="G8" s="34" t="n"/>
-      <c r="H8" s="34" t="n"/>
-      <c r="I8" s="34" t="n"/>
-      <c r="J8" s="34" t="inlineStr">
+      <c r="H8" s="42" t="n"/>
+      <c r="I8" s="42" t="n"/>
+      <c r="J8" s="42" t="n"/>
+      <c r="K8" s="42" t="inlineStr">
         <is>
           <t>964,346</t>
         </is>
       </c>
-      <c r="K8" s="34" t="inlineStr">
+      <c r="L8" s="42" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="L8" s="34" t="n"/>
-      <c r="M8" s="34" t="n"/>
-      <c r="N8" s="34" t="n"/>
-      <c r="O8" s="35" t="inlineStr">
+      <c r="M8" s="42" t="n"/>
+      <c r="N8" s="42" t="n"/>
+      <c r="O8" s="42" t="n"/>
+      <c r="P8" s="43" t="inlineStr">
         <is>
           <t>1,500,000</t>
         </is>
       </c>
     </row>
     <row r="9" ht="13" customHeight="1">
-      <c r="A9" s="36" t="n"/>
-      <c r="B9" s="37" t="n"/>
-      <c r="C9" s="20" t="n"/>
-      <c r="D9" s="38" t="inlineStr">
+      <c r="A9" s="44" t="inlineStr">
+        <is>
+          <t>元決済</t>
+        </is>
+      </c>
+      <c r="B9" s="45" t="inlineStr">
+        <is>
+          <t>実績粗利     14,278,312 率 43</t>
+        </is>
+      </c>
+      <c r="C9" s="46" t="inlineStr">
+        <is>
+          <t>実績売上     33,173,241</t>
+        </is>
+      </c>
+      <c r="D9" s="26" t="n"/>
+      <c r="E9" s="47" t="inlineStr">
         <is>
           <t>95.8</t>
         </is>
       </c>
-      <c r="E9" s="39" t="n"/>
-      <c r="F9" s="39" t="inlineStr">
-        <is>
-          <t>97</t>
-        </is>
-      </c>
-      <c r="G9" s="39" t="n"/>
-      <c r="H9" s="39" t="n"/>
-      <c r="I9" s="39" t="n"/>
-      <c r="J9" s="39" t="inlineStr">
+      <c r="F9" s="48" t="n"/>
+      <c r="G9" s="48" t="inlineStr">
+        <is>
+          <t>97%</t>
+        </is>
+      </c>
+      <c r="H9" s="48" t="n"/>
+      <c r="I9" s="48" t="n"/>
+      <c r="J9" s="48" t="n"/>
+      <c r="K9" s="48" t="inlineStr">
         <is>
           <t>0.4</t>
         </is>
       </c>
-      <c r="K9" s="39" t="inlineStr">
+      <c r="L9" s="48" t="inlineStr">
         <is>
           <t>0.0</t>
         </is>
       </c>
-      <c r="L9" s="39" t="n"/>
-      <c r="M9" s="39" t="n"/>
-      <c r="N9" s="39" t="n"/>
-      <c r="O9" s="40" t="inlineStr">
+      <c r="M9" s="48" t="n"/>
+      <c r="N9" s="48" t="n"/>
+      <c r="O9" s="48" t="n"/>
+      <c r="P9" s="49" t="inlineStr">
         <is>
           <t>3,333,333</t>
         </is>
       </c>
     </row>
     <row r="10" ht="13" customHeight="1">
-      <c r="A10" s="36" t="n"/>
-      <c r="B10" s="37" t="inlineStr">
+      <c r="A10" s="44" t="n"/>
+      <c r="B10" s="45" t="inlineStr">
+        <is>
+          <t>目標粗利     18,000,000 率 45</t>
+        </is>
+      </c>
+      <c r="C10" s="46" t="inlineStr">
+        <is>
+          <t>目標売上     40,000,000</t>
+        </is>
+      </c>
+      <c r="D10" s="50" t="inlineStr">
         <is>
           <t>累計</t>
         </is>
       </c>
-      <c r="C10" s="41" t="inlineStr">
-        <is>
-          <t>累計</t>
-        </is>
-      </c>
-      <c r="D10" s="42" t="inlineStr">
+      <c r="E10" s="51" t="inlineStr">
         <is>
           <t>15,871,447</t>
         </is>
       </c>
-      <c r="E10" s="43" t="inlineStr">
+      <c r="F10" s="52" t="inlineStr">
         <is>
           <t>42.5</t>
         </is>
       </c>
-      <c r="F10" s="43" t="inlineStr">
+      <c r="G10" s="52" t="inlineStr">
         <is>
           <t>37,355,692</t>
         </is>
       </c>
-      <c r="G10" s="43" t="n"/>
-      <c r="H10" s="43" t="n"/>
-      <c r="I10" s="43" t="n"/>
-      <c r="J10" s="43" t="inlineStr">
+      <c r="H10" s="52" t="n"/>
+      <c r="I10" s="52" t="n"/>
+      <c r="J10" s="52" t="n"/>
+      <c r="K10" s="52" t="inlineStr">
         <is>
           <t>1,299,717</t>
         </is>
       </c>
-      <c r="K10" s="43" t="inlineStr">
+      <c r="L10" s="52" t="inlineStr">
         <is>
           <t>1,197</t>
         </is>
       </c>
-      <c r="L10" s="43" t="n"/>
-      <c r="M10" s="43" t="n"/>
-      <c r="N10" s="43" t="n"/>
-      <c r="O10" s="44" t="inlineStr">
+      <c r="M10" s="52" t="n"/>
+      <c r="N10" s="52" t="n"/>
+      <c r="O10" s="52" t="n"/>
+      <c r="P10" s="53" t="inlineStr">
         <is>
           <t>16,500,000</t>
         </is>
       </c>
     </row>
     <row r="11" ht="13" customHeight="1">
-      <c r="A11" s="45" t="n"/>
-      <c r="B11" s="46" t="n"/>
-      <c r="C11" s="20" t="n"/>
-      <c r="D11" s="38" t="inlineStr">
+      <c r="A11" s="54" t="n"/>
+      <c r="B11" s="55" t="n"/>
+      <c r="C11" s="56" t="inlineStr">
+        <is>
+          <t>目標在庫     1,400,000</t>
+        </is>
+      </c>
+      <c r="D11" s="26" t="n"/>
+      <c r="E11" s="47" t="inlineStr">
         <is>
           <t>96.2</t>
         </is>
       </c>
-      <c r="E11" s="39" t="n"/>
-      <c r="F11" s="39" t="inlineStr">
+      <c r="F11" s="48" t="n"/>
+      <c r="G11" s="48" t="inlineStr">
         <is>
           <t>101.8</t>
         </is>
       </c>
-      <c r="G11" s="39" t="n"/>
-      <c r="H11" s="39" t="n"/>
-      <c r="I11" s="39" t="n"/>
-      <c r="J11" s="39" t="n"/>
-      <c r="K11" s="39" t="n"/>
-      <c r="L11" s="39" t="n"/>
-      <c r="M11" s="39" t="n"/>
-      <c r="N11" s="39" t="n"/>
-      <c r="O11" s="40" t="inlineStr">
+      <c r="H11" s="48" t="n"/>
+      <c r="I11" s="48" t="n"/>
+      <c r="J11" s="48" t="n"/>
+      <c r="K11" s="48" t="n"/>
+      <c r="L11" s="48" t="n"/>
+      <c r="M11" s="48" t="n"/>
+      <c r="N11" s="48" t="n"/>
+      <c r="O11" s="48" t="n"/>
+      <c r="P11" s="49" t="inlineStr">
         <is>
           <t>36,666,667</t>
         </is>
       </c>
     </row>
     <row r="12" ht="13" customHeight="1">
-      <c r="A12" s="30" t="inlineStr">
-        <is>
-          <t>シ50
-元決済
-＋円</t>
-        </is>
-      </c>
-      <c r="B12" s="31" t="inlineStr">
+      <c r="A12" s="37" t="inlineStr">
+        <is>
+          <t>シ50</t>
+        </is>
+      </c>
+      <c r="B12" s="38" t="inlineStr">
+        <is>
+          <t>(株)ジュン</t>
+        </is>
+      </c>
+      <c r="C12" s="39" t="n"/>
+      <c r="D12" s="40" t="inlineStr">
         <is>
           <t>当月</t>
         </is>
       </c>
-      <c r="C12" s="32" t="inlineStr">
-        <is>
-          <t>当月</t>
-        </is>
-      </c>
-      <c r="D12" s="33" t="inlineStr">
+      <c r="E12" s="41" t="inlineStr">
         <is>
           <t>7,445,009</t>
         </is>
       </c>
-      <c r="E12" s="34" t="inlineStr">
+      <c r="F12" s="42" t="inlineStr">
         <is>
           <t>36.7</t>
         </is>
       </c>
-      <c r="F12" s="34" t="inlineStr">
+      <c r="G12" s="42" t="inlineStr">
         <is>
           <t>20,258,139</t>
         </is>
       </c>
-      <c r="G12" s="34" t="n"/>
-      <c r="H12" s="34" t="inlineStr">
-        <is>
-          <t>33.4</t>
-        </is>
-      </c>
-      <c r="I12" s="34" t="inlineStr">
+      <c r="H12" s="42" t="n"/>
+      <c r="I12" s="42" t="n"/>
+      <c r="J12" s="42" t="inlineStr">
         <is>
           <t>159,000</t>
         </is>
       </c>
-      <c r="J12" s="34" t="inlineStr">
+      <c r="K12" s="42" t="inlineStr">
         <is>
           <t>32,234,375</t>
         </is>
       </c>
-      <c r="K12" s="34" t="inlineStr">
+      <c r="L12" s="42" t="inlineStr">
         <is>
           <t>362,832</t>
         </is>
       </c>
-      <c r="L12" s="34" t="n"/>
-      <c r="M12" s="34" t="n"/>
-      <c r="N12" s="34" t="n"/>
-      <c r="O12" s="35" t="inlineStr">
+      <c r="M12" s="42" t="n"/>
+      <c r="N12" s="42" t="n"/>
+      <c r="O12" s="42" t="n"/>
+      <c r="P12" s="43" t="inlineStr">
         <is>
           <t>10,484,250</t>
         </is>
       </c>
     </row>
     <row r="13" ht="13" customHeight="1">
-      <c r="A13" s="36" t="n"/>
-      <c r="B13" s="37" t="n"/>
-      <c r="C13" s="20" t="n"/>
-      <c r="D13" s="38" t="inlineStr">
+      <c r="A13" s="44" t="inlineStr">
+        <is>
+          <t>元決済</t>
+        </is>
+      </c>
+      <c r="B13" s="45" t="inlineStr">
+        <is>
+          <t>実績粗利     129,686,062 率 35</t>
+        </is>
+      </c>
+      <c r="C13" s="46" t="inlineStr">
+        <is>
+          <t>実績売上     372,927,122</t>
+        </is>
+      </c>
+      <c r="D13" s="26" t="n"/>
+      <c r="E13" s="47" t="inlineStr">
         <is>
           <t>71.0</t>
         </is>
       </c>
-      <c r="E13" s="39" t="n"/>
-      <c r="F13" s="39" t="inlineStr">
+      <c r="F13" s="48" t="n"/>
+      <c r="G13" s="48" t="inlineStr">
         <is>
           <t>72.1</t>
         </is>
       </c>
-      <c r="G13" s="39" t="n"/>
-      <c r="H13" s="39" t="n"/>
-      <c r="I13" s="39" t="inlineStr">
+      <c r="H13" s="48" t="n"/>
+      <c r="I13" s="48" t="inlineStr">
+        <is>
+          <t>33.4</t>
+        </is>
+      </c>
+      <c r="J13" s="48" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="J13" s="39" t="inlineStr">
+      <c r="K13" s="48" t="inlineStr">
         <is>
           <t>2.4</t>
         </is>
       </c>
-      <c r="K13" s="39" t="inlineStr">
+      <c r="L13" s="48" t="inlineStr">
         <is>
           <t>3.4</t>
         </is>
       </c>
-      <c r="L13" s="39" t="n"/>
-      <c r="M13" s="39" t="n"/>
-      <c r="N13" s="39" t="n"/>
-      <c r="O13" s="40" t="inlineStr">
+      <c r="M13" s="48" t="n"/>
+      <c r="N13" s="48" t="n"/>
+      <c r="O13" s="48" t="n"/>
+      <c r="P13" s="49" t="inlineStr">
         <is>
           <t>28,083,333</t>
         </is>
       </c>
     </row>
     <row r="14" ht="13" customHeight="1">
-      <c r="A14" s="36" t="n"/>
-      <c r="B14" s="37" t="inlineStr">
+      <c r="A14" s="44" t="inlineStr">
+        <is>
+          <t>＋円</t>
+        </is>
+      </c>
+      <c r="B14" s="45" t="inlineStr">
+        <is>
+          <t>目標粗利     141,500,000 率 37</t>
+        </is>
+      </c>
+      <c r="C14" s="46" t="inlineStr">
+        <is>
+          <t>目標売上     380,000,000</t>
+        </is>
+      </c>
+      <c r="D14" s="50" t="inlineStr">
         <is>
           <t>累計</t>
         </is>
       </c>
-      <c r="C14" s="41" t="inlineStr">
-        <is>
-          <t>累計</t>
-        </is>
-      </c>
-      <c r="D14" s="42" t="inlineStr">
+      <c r="E14" s="51" t="inlineStr">
         <is>
           <t>118,838,933</t>
         </is>
       </c>
-      <c r="E14" s="43" t="inlineStr">
+      <c r="F14" s="52" t="inlineStr">
         <is>
           <t>36.5</t>
         </is>
       </c>
-      <c r="F14" s="43" t="inlineStr">
+      <c r="G14" s="52" t="inlineStr">
         <is>
           <t>325,005,928</t>
         </is>
       </c>
-      <c r="G14" s="43" t="n"/>
-      <c r="H14" s="43" t="inlineStr">
-        <is>
-          <t>33.5</t>
-        </is>
-      </c>
-      <c r="I14" s="43" t="inlineStr">
+      <c r="H14" s="52" t="n"/>
+      <c r="I14" s="52" t="n"/>
+      <c r="J14" s="52" t="inlineStr">
         <is>
           <t>2,590,000</t>
         </is>
       </c>
-      <c r="J14" s="43" t="inlineStr">
+      <c r="K14" s="52" t="inlineStr">
         <is>
           <t>28,710,339</t>
         </is>
       </c>
-      <c r="K14" s="43" t="inlineStr">
+      <c r="L14" s="52" t="inlineStr">
         <is>
           <t>464,595</t>
         </is>
       </c>
-      <c r="L14" s="43" t="n"/>
-      <c r="M14" s="43" t="n"/>
-      <c r="N14" s="43" t="n"/>
-      <c r="O14" s="44" t="inlineStr">
+      <c r="M14" s="52" t="n"/>
+      <c r="N14" s="52" t="n"/>
+      <c r="O14" s="52" t="n"/>
+      <c r="P14" s="53" t="inlineStr">
         <is>
           <t>129,574,640</t>
         </is>
       </c>
     </row>
     <row r="15" ht="13" customHeight="1">
-      <c r="A15" s="47" t="n"/>
-      <c r="B15" s="48" t="n"/>
-      <c r="C15" s="49" t="n"/>
-      <c r="D15" s="50" t="inlineStr">
+      <c r="A15" s="57" t="n"/>
+      <c r="B15" s="58" t="n"/>
+      <c r="C15" s="59" t="inlineStr">
+        <is>
+          <t>目標在庫     29,400,000</t>
+        </is>
+      </c>
+      <c r="D15" s="60" t="n"/>
+      <c r="E15" s="61" t="inlineStr">
         <is>
           <t>91.7</t>
         </is>
       </c>
-      <c r="E15" s="51" t="n"/>
-      <c r="F15" s="51" t="inlineStr">
+      <c r="F15" s="62" t="n"/>
+      <c r="G15" s="62" t="inlineStr">
         <is>
           <t>93.4</t>
         </is>
       </c>
-      <c r="G15" s="51" t="n"/>
-      <c r="H15" s="51" t="n"/>
-      <c r="I15" s="51" t="inlineStr">
+      <c r="H15" s="62" t="n"/>
+      <c r="I15" s="62" t="inlineStr">
+        <is>
+          <t>33.5</t>
+        </is>
+      </c>
+      <c r="J15" s="62" t="inlineStr">
         <is>
           <t>68,400</t>
         </is>
       </c>
-      <c r="J15" s="51" t="n"/>
-      <c r="K15" s="51" t="n"/>
-      <c r="L15" s="51" t="n"/>
-      <c r="M15" s="51" t="n"/>
-      <c r="N15" s="51" t="n"/>
-      <c r="O15" s="52" t="inlineStr">
+      <c r="K15" s="62" t="n"/>
+      <c r="L15" s="62" t="n"/>
+      <c r="M15" s="62" t="n"/>
+      <c r="N15" s="62" t="n"/>
+      <c r="O15" s="62" t="n"/>
+      <c r="P15" s="63" t="inlineStr">
         <is>
           <t>347,946,667</t>
         </is>
       </c>
     </row>
     <row r="16" ht="13" customHeight="1">
-      <c r="A16" s="53" t="n"/>
-      <c r="B16" s="54" t="inlineStr">
+      <c r="A16" s="64" t="n"/>
+      <c r="B16" s="65" t="inlineStr">
+        <is>
+          <t>【大久保・関谷・金柿　円合計】</t>
+        </is>
+      </c>
+      <c r="C16" s="66" t="n"/>
+      <c r="D16" s="67" t="inlineStr">
         <is>
           <t>当月</t>
         </is>
       </c>
-      <c r="C16" s="55" t="inlineStr">
-        <is>
-          <t>当月</t>
-        </is>
-      </c>
-      <c r="D16" s="56" t="inlineStr">
+      <c r="E16" s="68" t="inlineStr">
         <is>
           <t>6,008,094</t>
         </is>
       </c>
-      <c r="E16" s="57" t="inlineStr">
+      <c r="F16" s="69" t="inlineStr">
         <is>
           <t>35.2</t>
         </is>
       </c>
-      <c r="F16" s="57" t="inlineStr">
+      <c r="G16" s="69" t="inlineStr">
         <is>
           <t>17,024,012</t>
         </is>
       </c>
-      <c r="G16" s="57" t="inlineStr">
+      <c r="H16" s="69" t="inlineStr">
         <is>
           <t>8,500,080</t>
         </is>
       </c>
-      <c r="H16" s="57" t="inlineStr">
+      <c r="I16" s="69" t="inlineStr">
         <is>
           <t>104,736</t>
         </is>
       </c>
-      <c r="I16" s="57" t="n"/>
-      <c r="J16" s="57" t="inlineStr">
+      <c r="J16" s="69" t="n"/>
+      <c r="K16" s="69" t="inlineStr">
         <is>
           <t>31,270,029</t>
         </is>
       </c>
-      <c r="K16" s="57" t="inlineStr">
+      <c r="L16" s="69" t="inlineStr">
         <is>
           <t>362,832</t>
         </is>
       </c>
-      <c r="L16" s="57" t="inlineStr">
+      <c r="M16" s="69" t="inlineStr">
         <is>
           <t>2,519,776</t>
         </is>
       </c>
-      <c r="M16" s="57" t="inlineStr">
+      <c r="N16" s="69" t="inlineStr">
         <is>
           <t>483</t>
         </is>
       </c>
-      <c r="N16" s="57" t="inlineStr">
+      <c r="O16" s="69" t="inlineStr">
         <is>
           <t>411,042</t>
         </is>
       </c>
-      <c r="O16" s="58" t="inlineStr">
+      <c r="P16" s="70" t="inlineStr">
         <is>
           <t>8,984,250</t>
         </is>
       </c>
     </row>
     <row r="17" ht="13" customHeight="1">
-      <c r="A17" s="59" t="n"/>
-      <c r="B17" s="19" t="n"/>
-      <c r="C17" s="20" t="n"/>
-      <c r="D17" s="21" t="inlineStr">
+      <c r="A17" s="71" t="n"/>
+      <c r="B17" s="24" t="inlineStr">
+        <is>
+          <t>実績粗利     115,407,750 率 34</t>
+        </is>
+      </c>
+      <c r="C17" s="25" t="inlineStr">
+        <is>
+          <t>実績売上     339,753,881</t>
+        </is>
+      </c>
+      <c r="D17" s="26" t="n"/>
+      <c r="E17" s="27" t="inlineStr">
         <is>
           <t>66.8</t>
         </is>
       </c>
-      <c r="E17" s="22" t="n"/>
-      <c r="F17" s="22" t="inlineStr">
+      <c r="F17" s="28" t="n"/>
+      <c r="G17" s="28" t="inlineStr">
         <is>
           <t>68.7</t>
         </is>
       </c>
-      <c r="G17" s="22" t="inlineStr">
+      <c r="H17" s="28" t="inlineStr">
         <is>
           <t>49.9</t>
         </is>
       </c>
-      <c r="H17" s="22" t="n"/>
-      <c r="I17" s="22" t="n"/>
-      <c r="J17" s="22" t="inlineStr">
+      <c r="I17" s="28" t="n"/>
+      <c r="J17" s="28" t="n"/>
+      <c r="K17" s="28" t="inlineStr">
         <is>
           <t>2.7</t>
         </is>
       </c>
-      <c r="K17" s="22" t="inlineStr">
+      <c r="L17" s="28" t="inlineStr">
         <is>
           <t>3.9</t>
         </is>
       </c>
-      <c r="L17" s="22" t="inlineStr">
+      <c r="M17" s="28" t="inlineStr">
         <is>
           <t>674,476</t>
         </is>
       </c>
-      <c r="M17" s="22" t="inlineStr">
+      <c r="N17" s="28" t="inlineStr">
         <is>
           <t>609,174</t>
         </is>
       </c>
-      <c r="N17" s="22" t="inlineStr">
+      <c r="O17" s="28" t="inlineStr">
         <is>
           <t>93,840</t>
         </is>
       </c>
-      <c r="O17" s="60" t="inlineStr">
+      <c r="P17" s="72" t="inlineStr">
         <is>
           <t>24,750,000</t>
         </is>
       </c>
     </row>
     <row r="18" ht="13" customHeight="1">
-      <c r="A18" s="59" t="n"/>
-      <c r="B18" s="19" t="inlineStr">
+      <c r="A18" s="71" t="n"/>
+      <c r="B18" s="24" t="inlineStr">
+        <is>
+          <t>目標粗利     123,500,000 率 36</t>
+        </is>
+      </c>
+      <c r="C18" s="25" t="inlineStr">
+        <is>
+          <t>目標売上     340,000,000</t>
+        </is>
+      </c>
+      <c r="D18" s="26" t="inlineStr">
         <is>
           <t>累計</t>
         </is>
       </c>
-      <c r="C18" s="20" t="inlineStr">
-        <is>
-          <t>累計</t>
-        </is>
-      </c>
-      <c r="D18" s="24" t="inlineStr">
+      <c r="E18" s="30" t="inlineStr">
         <is>
           <t>102,967,486</t>
         </is>
       </c>
-      <c r="E18" s="25" t="inlineStr">
+      <c r="F18" s="31" t="inlineStr">
         <is>
           <t>35.7</t>
         </is>
       </c>
-      <c r="F18" s="25" t="inlineStr">
+      <c r="G18" s="31" t="inlineStr">
         <is>
           <t>287,650,236</t>
         </is>
       </c>
-      <c r="G18" s="25" t="inlineStr">
+      <c r="H18" s="31" t="inlineStr">
         <is>
           <t>182,124,664</t>
         </is>
       </c>
-      <c r="H18" s="25" t="inlineStr">
+      <c r="I18" s="31" t="inlineStr">
         <is>
           <t>1,118,068</t>
         </is>
       </c>
-      <c r="I18" s="25" t="n"/>
-      <c r="J18" s="25" t="inlineStr">
+      <c r="J18" s="31" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="K18" s="31" t="inlineStr">
         <is>
           <t>27,410,622</t>
         </is>
       </c>
-      <c r="K18" s="25" t="inlineStr">
+      <c r="L18" s="31" t="inlineStr">
         <is>
           <t>463,398</t>
         </is>
       </c>
-      <c r="L18" s="25" t="inlineStr">
+      <c r="M18" s="31" t="inlineStr">
         <is>
           <t>35,835,714</t>
         </is>
       </c>
-      <c r="M18" s="25" t="inlineStr">
+      <c r="N18" s="31" t="inlineStr">
         <is>
           <t>6,601</t>
         </is>
       </c>
-      <c r="N18" s="25" t="inlineStr">
+      <c r="O18" s="31" t="inlineStr">
         <is>
           <t>5,135,954</t>
         </is>
       </c>
-      <c r="O18" s="61" t="inlineStr">
+      <c r="P18" s="73" t="inlineStr">
         <is>
           <t>113,074,640</t>
         </is>
       </c>
     </row>
     <row r="19" ht="13" customHeight="1">
-      <c r="A19" s="59" t="n"/>
-      <c r="B19" s="28" t="n"/>
-      <c r="C19" s="20" t="n"/>
-      <c r="D19" s="21" t="inlineStr">
+      <c r="A19" s="71" t="n"/>
+      <c r="B19" s="34" t="n"/>
+      <c r="C19" s="35" t="inlineStr">
+        <is>
+          <t>目標在庫     28,000,000</t>
+        </is>
+      </c>
+      <c r="D19" s="26" t="n"/>
+      <c r="E19" s="27" t="inlineStr">
         <is>
           <t>91.0</t>
         </is>
       </c>
-      <c r="E19" s="22" t="inlineStr">
+      <c r="F19" s="28" t="inlineStr">
         <is>
           <t>34.6</t>
         </is>
       </c>
-      <c r="F19" s="22" t="inlineStr">
+      <c r="G19" s="28" t="inlineStr">
         <is>
           <t>92.4</t>
         </is>
       </c>
-      <c r="G19" s="22" t="inlineStr">
+      <c r="H19" s="28" t="inlineStr">
         <is>
           <t>63.3</t>
         </is>
       </c>
-      <c r="H19" s="22" t="n"/>
-      <c r="I19" s="22" t="n"/>
-      <c r="J19" s="22" t="inlineStr">
+      <c r="I19" s="28" t="n"/>
+      <c r="J19" s="28" t="n"/>
+      <c r="K19" s="28" t="inlineStr">
         <is>
           <t>0.0</t>
         </is>
       </c>
-      <c r="K19" s="22" t="n"/>
-      <c r="L19" s="22" t="inlineStr">
+      <c r="L19" s="28" t="n"/>
+      <c r="M19" s="28" t="inlineStr">
         <is>
           <t>10,973,554</t>
         </is>
       </c>
-      <c r="M19" s="22" t="inlineStr">
+      <c r="N19" s="28" t="inlineStr">
         <is>
           <t>12,086,717</t>
         </is>
       </c>
-      <c r="N19" s="22" t="inlineStr">
+      <c r="O19" s="28" t="inlineStr">
         <is>
           <t>1,881,400</t>
         </is>
       </c>
-      <c r="O19" s="60" t="inlineStr">
+      <c r="P19" s="72" t="inlineStr">
         <is>
           <t>311,280,000</t>
         </is>
       </c>
     </row>
     <row r="20" ht="13" customHeight="1">
-      <c r="A20" s="62" t="n"/>
-      <c r="B20" s="31" t="inlineStr">
+      <c r="A20" s="74" t="n"/>
+      <c r="B20" s="38" t="inlineStr">
+        <is>
+          <t>【大久保・関谷・金柿　元合計】</t>
+        </is>
+      </c>
+      <c r="C20" s="39" t="n"/>
+      <c r="D20" s="40" t="inlineStr">
         <is>
           <t>当月</t>
         </is>
       </c>
-      <c r="C20" s="32" t="inlineStr">
-        <is>
-          <t>当月</t>
-        </is>
-      </c>
-      <c r="D20" s="33" t="inlineStr">
+      <c r="E20" s="41" t="inlineStr">
         <is>
           <t>1,436,915</t>
         </is>
       </c>
-      <c r="E20" s="34" t="inlineStr">
+      <c r="F20" s="42" t="inlineStr">
         <is>
           <t>44.4</t>
         </is>
       </c>
-      <c r="F20" s="34" t="inlineStr">
+      <c r="G20" s="42" t="inlineStr">
         <is>
           <t>3,234,127</t>
         </is>
       </c>
-      <c r="G20" s="34" t="n"/>
-      <c r="H20" s="34" t="n"/>
-      <c r="I20" s="34" t="n"/>
-      <c r="J20" s="34" t="inlineStr">
+      <c r="H20" s="42" t="n"/>
+      <c r="I20" s="42" t="n"/>
+      <c r="J20" s="42" t="n"/>
+      <c r="K20" s="42" t="inlineStr">
         <is>
           <t>964,346</t>
         </is>
       </c>
-      <c r="K20" s="34" t="inlineStr">
+      <c r="L20" s="42" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="L20" s="34" t="n"/>
-      <c r="M20" s="34" t="n"/>
-      <c r="N20" s="34" t="n"/>
-      <c r="O20" s="63" t="inlineStr">
+      <c r="M20" s="42" t="n"/>
+      <c r="N20" s="42" t="n"/>
+      <c r="O20" s="42" t="n"/>
+      <c r="P20" s="75" t="inlineStr">
         <is>
           <t>1,500,000</t>
         </is>
       </c>
     </row>
     <row r="21" ht="13" customHeight="1">
-      <c r="A21" s="62" t="n"/>
-      <c r="B21" s="37" t="n"/>
-      <c r="C21" s="20" t="n"/>
-      <c r="D21" s="38" t="inlineStr">
+      <c r="A21" s="74" t="n"/>
+      <c r="B21" s="45" t="inlineStr">
+        <is>
+          <t>実績粗利     14,278,312 率 43</t>
+        </is>
+      </c>
+      <c r="C21" s="46" t="inlineStr">
+        <is>
+          <t>実績売上     33,173,241</t>
+        </is>
+      </c>
+      <c r="D21" s="26" t="n"/>
+      <c r="E21" s="47" t="inlineStr">
         <is>
           <t>95.7</t>
         </is>
       </c>
-      <c r="E21" s="39" t="n"/>
-      <c r="F21" s="39" t="inlineStr">
+      <c r="F21" s="48" t="n"/>
+      <c r="G21" s="48" t="inlineStr">
         <is>
           <t>97.0</t>
         </is>
       </c>
-      <c r="G21" s="39" t="n"/>
-      <c r="H21" s="39" t="n"/>
-      <c r="I21" s="39" t="n"/>
-      <c r="J21" s="39" t="inlineStr">
+      <c r="H21" s="48" t="n"/>
+      <c r="I21" s="48" t="n"/>
+      <c r="J21" s="48" t="n"/>
+      <c r="K21" s="48" t="inlineStr">
         <is>
           <t>0.4</t>
         </is>
       </c>
-      <c r="K21" s="39" t="inlineStr">
+      <c r="L21" s="48" t="inlineStr">
         <is>
           <t>0.0</t>
         </is>
       </c>
-      <c r="L21" s="39" t="n"/>
-      <c r="M21" s="39" t="n"/>
-      <c r="N21" s="39" t="n"/>
-      <c r="O21" s="64" t="inlineStr">
+      <c r="M21" s="48" t="n"/>
+      <c r="N21" s="48" t="n"/>
+      <c r="O21" s="48" t="n"/>
+      <c r="P21" s="76" t="inlineStr">
         <is>
           <t>3,333,333</t>
         </is>
       </c>
     </row>
     <row r="22" ht="13" customHeight="1">
-      <c r="A22" s="62" t="n"/>
-      <c r="B22" s="37" t="inlineStr">
+      <c r="A22" s="74" t="n"/>
+      <c r="B22" s="45" t="inlineStr">
+        <is>
+          <t>目標粗利     18,000,000 率 45</t>
+        </is>
+      </c>
+      <c r="C22" s="46" t="inlineStr">
+        <is>
+          <t>目標売上     40,000,000</t>
+        </is>
+      </c>
+      <c r="D22" s="50" t="inlineStr">
         <is>
           <t>累計</t>
         </is>
       </c>
-      <c r="C22" s="41" t="inlineStr">
-        <is>
-          <t>累計</t>
-        </is>
-      </c>
-      <c r="D22" s="42" t="inlineStr">
+      <c r="E22" s="51" t="inlineStr">
         <is>
           <t>15,871,447</t>
         </is>
       </c>
-      <c r="E22" s="43" t="inlineStr">
+      <c r="F22" s="52" t="inlineStr">
         <is>
           <t>42.4</t>
         </is>
       </c>
-      <c r="F22" s="43" t="inlineStr">
+      <c r="G22" s="52" t="inlineStr">
         <is>
           <t>37,355,692</t>
         </is>
       </c>
-      <c r="G22" s="43" t="n"/>
-      <c r="H22" s="43" t="n"/>
-      <c r="I22" s="43" t="n"/>
-      <c r="J22" s="43" t="inlineStr">
+      <c r="H22" s="52" t="n"/>
+      <c r="I22" s="52" t="n"/>
+      <c r="J22" s="52" t="n"/>
+      <c r="K22" s="52" t="inlineStr">
         <is>
           <t>1,299,717</t>
         </is>
       </c>
-      <c r="K22" s="43" t="inlineStr">
+      <c r="L22" s="52" t="inlineStr">
         <is>
           <t>1,197</t>
         </is>
       </c>
-      <c r="L22" s="43" t="n"/>
-      <c r="M22" s="43" t="n"/>
-      <c r="N22" s="43" t="n"/>
-      <c r="O22" s="65" t="inlineStr">
+      <c r="M22" s="52" t="n"/>
+      <c r="N22" s="52" t="n"/>
+      <c r="O22" s="52" t="n"/>
+      <c r="P22" s="77" t="inlineStr">
         <is>
           <t>16,500,000</t>
         </is>
       </c>
     </row>
     <row r="23" ht="13" customHeight="1">
-      <c r="A23" s="62" t="n"/>
-      <c r="B23" s="46" t="n"/>
-      <c r="C23" s="20" t="n"/>
-      <c r="D23" s="38" t="inlineStr">
+      <c r="A23" s="74" t="n"/>
+      <c r="B23" s="55" t="n"/>
+      <c r="C23" s="56" t="inlineStr">
+        <is>
+          <t>目標在庫     1,400,000</t>
+        </is>
+      </c>
+      <c r="D23" s="26" t="n"/>
+      <c r="E23" s="47" t="inlineStr">
         <is>
           <t>96.1</t>
         </is>
       </c>
-      <c r="E23" s="39" t="n"/>
-      <c r="F23" s="39" t="inlineStr">
+      <c r="F23" s="48" t="n"/>
+      <c r="G23" s="48" t="inlineStr">
         <is>
           <t>101.8</t>
         </is>
       </c>
-      <c r="G23" s="39" t="n"/>
-      <c r="H23" s="39" t="n"/>
-      <c r="I23" s="39" t="n"/>
-      <c r="J23" s="39" t="n"/>
-      <c r="K23" s="39" t="n"/>
-      <c r="L23" s="39" t="n"/>
-      <c r="M23" s="39" t="n"/>
-      <c r="N23" s="39" t="n"/>
-      <c r="O23" s="64" t="inlineStr">
+      <c r="H23" s="48" t="n"/>
+      <c r="I23" s="48" t="n"/>
+      <c r="J23" s="48" t="n"/>
+      <c r="K23" s="48" t="n"/>
+      <c r="L23" s="48" t="n"/>
+      <c r="M23" s="48" t="n"/>
+      <c r="N23" s="48" t="n"/>
+      <c r="O23" s="48" t="n"/>
+      <c r="P23" s="76" t="inlineStr">
         <is>
           <t>36,666,667</t>
         </is>
       </c>
     </row>
     <row r="24" ht="13" customHeight="1">
-      <c r="A24" s="62" t="n"/>
-      <c r="B24" s="31" t="inlineStr">
+      <c r="A24" s="74" t="n"/>
+      <c r="B24" s="38" t="inlineStr">
+        <is>
+          <t>【大久保・関谷・金柿　円＋元　合計】</t>
+        </is>
+      </c>
+      <c r="C24" s="39" t="n"/>
+      <c r="D24" s="40" t="inlineStr">
         <is>
           <t>当月</t>
         </is>
       </c>
-      <c r="C24" s="32" t="inlineStr">
-        <is>
-          <t>当月</t>
-        </is>
-      </c>
-      <c r="D24" s="33" t="inlineStr">
+      <c r="E24" s="41" t="inlineStr">
         <is>
           <t>7,445,009</t>
         </is>
       </c>
-      <c r="E24" s="34" t="inlineStr">
+      <c r="F24" s="42" t="inlineStr">
         <is>
           <t>36.7</t>
         </is>
       </c>
-      <c r="F24" s="34" t="inlineStr">
+      <c r="G24" s="42" t="inlineStr">
         <is>
           <t>20,258,139</t>
         </is>
       </c>
-      <c r="G24" s="34" t="n"/>
-      <c r="H24" s="34" t="inlineStr">
-        <is>
-          <t>33.4</t>
-        </is>
-      </c>
-      <c r="I24" s="34" t="inlineStr">
+      <c r="H24" s="42" t="n"/>
+      <c r="I24" s="42" t="n"/>
+      <c r="J24" s="42" t="inlineStr">
         <is>
           <t>159,000</t>
         </is>
       </c>
-      <c r="J24" s="34" t="inlineStr">
+      <c r="K24" s="42" t="inlineStr">
         <is>
           <t>32,234,375</t>
         </is>
       </c>
-      <c r="K24" s="34" t="inlineStr">
+      <c r="L24" s="42" t="inlineStr">
         <is>
           <t>362,832</t>
         </is>
       </c>
-      <c r="L24" s="34" t="n"/>
-      <c r="M24" s="34" t="n"/>
-      <c r="N24" s="34" t="n"/>
-      <c r="O24" s="63" t="inlineStr">
+      <c r="M24" s="42" t="n"/>
+      <c r="N24" s="42" t="n"/>
+      <c r="O24" s="42" t="n"/>
+      <c r="P24" s="75" t="inlineStr">
         <is>
           <t>10,484,250</t>
         </is>
       </c>
     </row>
     <row r="25" ht="13" customHeight="1">
-      <c r="A25" s="62" t="n"/>
-      <c r="B25" s="37" t="n"/>
-      <c r="C25" s="20" t="n"/>
-      <c r="D25" s="38" t="inlineStr">
+      <c r="A25" s="74" t="n"/>
+      <c r="B25" s="45" t="inlineStr">
+        <is>
+          <t>実績粗利     129,686,062 率 35</t>
+        </is>
+      </c>
+      <c r="C25" s="46" t="inlineStr">
+        <is>
+          <t>実績売上     372,927,122</t>
+        </is>
+      </c>
+      <c r="D25" s="26" t="n"/>
+      <c r="E25" s="47" t="inlineStr">
         <is>
           <t>71.0</t>
         </is>
       </c>
-      <c r="E25" s="39" t="n"/>
-      <c r="F25" s="39" t="inlineStr">
+      <c r="F25" s="48" t="n"/>
+      <c r="G25" s="48" t="inlineStr">
         <is>
           <t>72.1</t>
         </is>
       </c>
-      <c r="G25" s="39" t="n"/>
-      <c r="H25" s="39" t="n"/>
-      <c r="I25" s="39" t="inlineStr">
+      <c r="H25" s="48" t="n"/>
+      <c r="I25" s="48" t="inlineStr">
+        <is>
+          <t>33.4</t>
+        </is>
+      </c>
+      <c r="J25" s="48" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="J25" s="39" t="inlineStr">
+      <c r="K25" s="48" t="inlineStr">
         <is>
           <t>2.4</t>
         </is>
       </c>
-      <c r="K25" s="39" t="inlineStr">
+      <c r="L25" s="48" t="inlineStr">
         <is>
           <t>3.4</t>
         </is>
       </c>
-      <c r="L25" s="39" t="n"/>
-      <c r="M25" s="39" t="n"/>
-      <c r="N25" s="39" t="n"/>
-      <c r="O25" s="64" t="inlineStr">
+      <c r="M25" s="48" t="n"/>
+      <c r="N25" s="48" t="n"/>
+      <c r="O25" s="48" t="n"/>
+      <c r="P25" s="76" t="inlineStr">
         <is>
           <t>28,083,333</t>
         </is>
       </c>
     </row>
     <row r="26" ht="13" customHeight="1">
-      <c r="A26" s="62" t="n"/>
-      <c r="B26" s="37" t="inlineStr">
+      <c r="A26" s="74" t="n"/>
+      <c r="B26" s="45" t="inlineStr">
+        <is>
+          <t>目標粗利     141,500,000 率 37</t>
+        </is>
+      </c>
+      <c r="C26" s="46" t="inlineStr">
+        <is>
+          <t>目標売上     380,000,000</t>
+        </is>
+      </c>
+      <c r="D26" s="50" t="inlineStr">
         <is>
           <t>累計</t>
         </is>
       </c>
-      <c r="C26" s="41" t="inlineStr">
-        <is>
-          <t>累計</t>
-        </is>
-      </c>
-      <c r="D26" s="42" t="inlineStr">
+      <c r="E26" s="51" t="inlineStr">
         <is>
           <t>118,838,933</t>
         </is>
       </c>
-      <c r="E26" s="43" t="inlineStr">
+      <c r="F26" s="52" t="inlineStr">
         <is>
           <t>36.5</t>
         </is>
       </c>
-      <c r="F26" s="43" t="inlineStr">
+      <c r="G26" s="52" t="inlineStr">
         <is>
           <t>325,005,928</t>
         </is>
       </c>
-      <c r="G26" s="43" t="n"/>
-      <c r="H26" s="43" t="inlineStr">
-        <is>
-          <t>33.5</t>
-        </is>
-      </c>
-      <c r="I26" s="43" t="inlineStr">
+      <c r="H26" s="52" t="n"/>
+      <c r="I26" s="52" t="n"/>
+      <c r="J26" s="52" t="inlineStr">
         <is>
           <t>2,590,000</t>
         </is>
       </c>
-      <c r="J26" s="43" t="inlineStr">
+      <c r="K26" s="52" t="inlineStr">
         <is>
           <t>28,710,339</t>
         </is>
       </c>
-      <c r="K26" s="43" t="inlineStr">
+      <c r="L26" s="52" t="inlineStr">
         <is>
           <t>464,595</t>
         </is>
       </c>
-      <c r="L26" s="43" t="n"/>
-      <c r="M26" s="43" t="n"/>
-      <c r="N26" s="43" t="n"/>
-      <c r="O26" s="65" t="inlineStr">
+      <c r="M26" s="52" t="n"/>
+      <c r="N26" s="52" t="n"/>
+      <c r="O26" s="52" t="n"/>
+      <c r="P26" s="77" t="inlineStr">
         <is>
           <t>129,574,640</t>
         </is>
       </c>
     </row>
     <row r="27" ht="13" customHeight="1">
-      <c r="A27" s="66" t="n"/>
-      <c r="B27" s="48" t="n"/>
-      <c r="C27" s="49" t="n"/>
-      <c r="D27" s="50" t="inlineStr">
+      <c r="A27" s="78" t="n"/>
+      <c r="B27" s="58" t="n"/>
+      <c r="C27" s="59" t="inlineStr">
+        <is>
+          <t>目標在庫     29,400,000</t>
+        </is>
+      </c>
+      <c r="D27" s="60" t="n"/>
+      <c r="E27" s="61" t="inlineStr">
         <is>
           <t>91.7</t>
         </is>
       </c>
-      <c r="E27" s="51" t="n"/>
-      <c r="F27" s="51" t="inlineStr">
+      <c r="F27" s="62" t="n"/>
+      <c r="G27" s="62" t="inlineStr">
         <is>
           <t>93.4</t>
         </is>
       </c>
-      <c r="G27" s="51" t="n"/>
-      <c r="H27" s="51" t="n"/>
-      <c r="I27" s="51" t="inlineStr">
+      <c r="H27" s="62" t="n"/>
+      <c r="I27" s="62" t="inlineStr">
+        <is>
+          <t>33.5</t>
+        </is>
+      </c>
+      <c r="J27" s="62" t="inlineStr">
         <is>
           <t>68,400</t>
         </is>
       </c>
-      <c r="J27" s="51" t="n"/>
-      <c r="K27" s="51" t="n"/>
-      <c r="L27" s="51" t="n"/>
-      <c r="M27" s="51" t="n"/>
-      <c r="N27" s="51" t="n"/>
-      <c r="O27" s="67" t="inlineStr">
+      <c r="K27" s="62" t="n"/>
+      <c r="L27" s="62" t="n"/>
+      <c r="M27" s="62" t="n"/>
+      <c r="N27" s="62" t="n"/>
+      <c r="O27" s="62" t="n"/>
+      <c r="P27" s="79" t="inlineStr">
         <is>
           <t>347,946,667</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="19">
-    <mergeCell ref="C4:C5"/>
-    <mergeCell ref="C20:C21"/>
+  <mergeCells count="20">
+    <mergeCell ref="E1:M1"/>
+    <mergeCell ref="N1:P1"/>
     <mergeCell ref="B2:B3"/>
-    <mergeCell ref="C10:C11"/>
-    <mergeCell ref="C16:C17"/>
-    <mergeCell ref="C26:C27"/>
-    <mergeCell ref="C22:C23"/>
-    <mergeCell ref="C12:C13"/>
+    <mergeCell ref="D2:D3"/>
+    <mergeCell ref="D4:D5"/>
+    <mergeCell ref="D16:D17"/>
     <mergeCell ref="A2:A3"/>
+    <mergeCell ref="D12:D13"/>
     <mergeCell ref="C2:C3"/>
-    <mergeCell ref="C8:C9"/>
-    <mergeCell ref="D1:L1"/>
+    <mergeCell ref="D24:D25"/>
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="D18:D19"/>
+    <mergeCell ref="D8:D9"/>
+    <mergeCell ref="D20:D21"/>
+    <mergeCell ref="D14:D15"/>
     <mergeCell ref="A16:A27"/>
-    <mergeCell ref="A1:C1"/>
-    <mergeCell ref="M1:O1"/>
-    <mergeCell ref="C6:C7"/>
-    <mergeCell ref="C24:C25"/>
-    <mergeCell ref="C18:C19"/>
-    <mergeCell ref="C14:C15"/>
+    <mergeCell ref="D10:D11"/>
+    <mergeCell ref="D26:D27"/>
+    <mergeCell ref="D6:D7"/>
+    <mergeCell ref="D22:D23"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>